<commit_message>
Updated main telemetry having participant IDs
</commit_message>
<xml_diff>
--- a/appendix/MGT - Experiment Research Data.xlsx
+++ b/appendix/MGT - Experiment Research Data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://edubuas.sharepoint.com/teams/2024-25MGT37/Shared Documents/General/Zeb de Roover - 256279/Working Files/Block C/CSV exports/Raw experiment data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GameDev\Projects\MGT VVVVVV\MGT-DDA-VVVVVV\appendix\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="28" documentId="11_B42B6CE3B7240B83D6683F6B04F51419A0DB2EFF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{28FD034E-622C-46D5-979E-1EC1633B6285}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C7766B3-0700-41EF-BF17-EF1293718EA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="705" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data Sheet" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="647" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="648" uniqueCount="246">
   <si>
     <t>Participant_id</t>
   </si>
@@ -828,6 +828,9 @@
   <si>
     <t>The 6 players were all people who played through the game's demo and uploaded their playthrough on YouTube.</t>
   </si>
+  <si>
+    <t>Participant ID</t>
+  </si>
 </sst>
 </file>
 
@@ -1051,22 +1054,6 @@
   </cellStyles>
   <dxfs count="8">
     <dxf>
-      <border>
-        <left style="thin">
-          <color rgb="FF5B3F86"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF5B3F86"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF5B3F86"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF5B3F86"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFF8F9FA"/>
@@ -1130,19 +1117,35 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF5B3F86"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF5B3F86"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF5B3F86"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF5B3F86"/>
+        </bottom>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="2">
     <tableStyle name="Questionnaire C-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="4"/>
-      <tableStyleElement type="headerRow" dxfId="7"/>
-      <tableStyleElement type="firstRowStripe" dxfId="6"/>
-      <tableStyleElement type="secondRowStripe" dxfId="5"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="7"/>
+      <tableStyleElement type="headerRow" dxfId="6"/>
+      <tableStyleElement type="firstRowStripe" dxfId="5"/>
+      <tableStyleElement type="secondRowStripe" dxfId="4"/>
     </tableStyle>
     <tableStyle name="Questionnaire E-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF01000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="0"/>
-      <tableStyleElement type="headerRow" dxfId="3"/>
-      <tableStyleElement type="firstRowStripe" dxfId="2"/>
-      <tableStyleElement type="secondRowStripe" dxfId="1"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="3"/>
+      <tableStyleElement type="headerRow" dxfId="2"/>
+      <tableStyleElement type="firstRowStripe" dxfId="1"/>
+      <tableStyleElement type="secondRowStripe" dxfId="0"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -17271,1902 +17274,2090 @@
     <tabColor rgb="FF1155CC"/>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:J71"/>
+  <dimension ref="A1:K71"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="21.88671875" customWidth="1"/>
-    <col min="2" max="2" width="17.88671875" customWidth="1"/>
-    <col min="3" max="3" width="11.109375" customWidth="1"/>
-    <col min="4" max="4" width="9.44140625" customWidth="1"/>
-    <col min="5" max="5" width="6.33203125" customWidth="1"/>
-    <col min="6" max="6" width="19.88671875" customWidth="1"/>
-    <col min="7" max="7" width="5.109375" customWidth="1"/>
-    <col min="8" max="8" width="9.44140625" customWidth="1"/>
-    <col min="9" max="9" width="255.6640625" customWidth="1"/>
+    <col min="2" max="2" width="21.88671875" customWidth="1"/>
+    <col min="3" max="3" width="17.88671875" customWidth="1"/>
+    <col min="4" max="4" width="11.109375" customWidth="1"/>
+    <col min="5" max="5" width="9.44140625" customWidth="1"/>
+    <col min="6" max="6" width="6.33203125" customWidth="1"/>
+    <col min="7" max="7" width="19.88671875" customWidth="1"/>
+    <col min="8" max="8" width="5.109375" customWidth="1"/>
+    <col min="9" max="9" width="9.44140625" customWidth="1"/>
+    <col min="10" max="10" width="255.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:10">
       <c r="A1" s="9" t="s">
+        <v>245</v>
+      </c>
+      <c r="B1" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="C1" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="D1" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="E1" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="F1" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="G1" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="H1" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="I1" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="J1" s="9" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
-      <c r="A2" s="10" t="s">
+    <row r="2" spans="1:10">
+      <c r="A2" s="10">
+        <v>1</v>
+      </c>
+      <c r="B2" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="C2" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="C2" s="10">
+      <c r="D2" s="10">
         <v>136</v>
       </c>
-      <c r="D2" s="11">
+      <c r="E2" s="11">
         <v>1.457175925925926E-2</v>
       </c>
-      <c r="E2" s="10">
+      <c r="F2" s="10">
         <v>63</v>
       </c>
-      <c r="F2" s="10" t="s">
+      <c r="G2" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="G2" s="10">
+      <c r="H2" s="10">
         <v>43</v>
       </c>
-      <c r="H2" s="10">
+      <c r="I2" s="10">
         <v>68.05</v>
       </c>
-      <c r="I2" s="10" t="s">
+      <c r="J2" s="10" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
-      <c r="A3" s="10" t="s">
+    <row r="3" spans="1:10">
+      <c r="A3" s="10">
+        <v>2</v>
+      </c>
+      <c r="B3" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="C3" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="C3" s="10">
+      <c r="D3" s="10">
         <v>142</v>
       </c>
-      <c r="D3" s="11">
+      <c r="E3" s="11">
         <v>1.0914351851851852E-2</v>
       </c>
-      <c r="E3" s="10">
+      <c r="F3" s="10">
         <v>63</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="G3" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="G3" s="10">
+      <c r="H3" s="10">
         <v>42</v>
       </c>
-      <c r="H3" s="10">
+      <c r="I3" s="10">
         <v>70.37</v>
       </c>
-      <c r="I3" s="10" t="s">
+      <c r="J3" s="10" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
-      <c r="A4" s="12" t="s">
+    <row r="4" spans="1:10">
+      <c r="A4" s="10">
+        <v>3</v>
+      </c>
+      <c r="B4" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="C4" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C4" s="12">
+      <c r="D4" s="12">
         <v>290</v>
       </c>
-      <c r="D4" s="13">
+      <c r="E4" s="13">
         <v>2.4189814814814813E-2</v>
       </c>
-      <c r="E4" s="12">
+      <c r="F4" s="12">
         <v>57</v>
       </c>
-      <c r="F4" s="12" t="s">
+      <c r="G4" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="G4" s="12">
+      <c r="H4" s="12">
         <v>40</v>
       </c>
-      <c r="H4" s="12">
+      <c r="I4" s="12">
         <v>64.08</v>
       </c>
-      <c r="I4" s="12" t="s">
+      <c r="J4" s="12" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
-      <c r="A5" s="12" t="s">
+    <row r="5" spans="1:10">
+      <c r="A5" s="10">
+        <v>4</v>
+      </c>
+      <c r="B5" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="C5" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C5" s="12">
+      <c r="D5" s="12">
         <v>126</v>
       </c>
-      <c r="D5" s="13">
+      <c r="E5" s="13">
         <v>1.3078703703703703E-2</v>
       </c>
-      <c r="E5" s="12">
+      <c r="F5" s="12">
         <v>63</v>
       </c>
-      <c r="F5" s="12" t="s">
+      <c r="G5" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="G5" s="12">
+      <c r="H5" s="12">
         <v>35</v>
       </c>
-      <c r="H5" s="12">
+      <c r="I5" s="12">
         <v>53.2</v>
       </c>
-      <c r="I5" s="12" t="s">
+      <c r="J5" s="12" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
-      <c r="A6" s="10" t="s">
+    <row r="6" spans="1:10">
+      <c r="A6" s="10">
+        <v>5</v>
+      </c>
+      <c r="B6" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="C6" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="C6" s="10">
+      <c r="D6" s="10">
         <v>131</v>
       </c>
-      <c r="D6" s="11">
+      <c r="E6" s="11">
         <v>1.0254629629629629E-2</v>
       </c>
-      <c r="E6" s="10">
+      <c r="F6" s="10">
         <v>63</v>
       </c>
-      <c r="F6" s="10" t="s">
+      <c r="G6" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="G6" s="10">
+      <c r="H6" s="10">
         <v>40</v>
       </c>
-      <c r="H6" s="10">
+      <c r="I6" s="10">
         <v>61.15</v>
       </c>
-      <c r="I6" s="10" t="s">
+      <c r="J6" s="10" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="7" spans="1:9">
-      <c r="A7" s="10" t="s">
+    <row r="7" spans="1:10">
+      <c r="A7" s="10">
+        <v>6</v>
+      </c>
+      <c r="B7" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="C7" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="C7" s="10">
+      <c r="D7" s="10">
         <v>247</v>
       </c>
-      <c r="D7" s="11">
+      <c r="E7" s="11">
         <v>1.758101851851852E-2</v>
       </c>
-      <c r="E7" s="10">
+      <c r="F7" s="10">
         <v>63</v>
       </c>
-      <c r="F7" s="10" t="s">
+      <c r="G7" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="G7" s="10">
+      <c r="H7" s="10">
         <v>43</v>
       </c>
-      <c r="H7" s="10">
+      <c r="I7" s="10">
         <v>55.85</v>
       </c>
-      <c r="I7" s="10" t="s">
+      <c r="J7" s="10" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
-      <c r="A8" s="12" t="s">
+    <row r="8" spans="1:10">
+      <c r="A8" s="10">
+        <v>7</v>
+      </c>
+      <c r="B8" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="C8" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C8" s="12">
+      <c r="D8" s="12">
         <v>97</v>
       </c>
-      <c r="D8" s="13">
+      <c r="E8" s="13">
         <v>1.1516203703703704E-2</v>
       </c>
-      <c r="E8" s="12">
+      <c r="F8" s="12">
         <v>63</v>
       </c>
-      <c r="F8" s="12" t="s">
+      <c r="G8" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="G8" s="12">
+      <c r="H8" s="12">
         <v>41</v>
       </c>
-      <c r="H8" s="12">
+      <c r="I8" s="12">
         <v>57.95</v>
       </c>
-      <c r="I8" s="12" t="s">
+      <c r="J8" s="12" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="9" spans="1:9">
-      <c r="A9" s="10" t="s">
+    <row r="9" spans="1:10">
+      <c r="A9" s="10">
+        <v>8</v>
+      </c>
+      <c r="B9" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="C9" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="C9" s="10">
+      <c r="D9" s="10">
         <v>153</v>
       </c>
-      <c r="D9" s="11">
+      <c r="E9" s="11">
         <v>1.2638888888888889E-2</v>
       </c>
-      <c r="E9" s="10">
+      <c r="F9" s="10">
         <v>63</v>
       </c>
-      <c r="F9" s="10" t="s">
+      <c r="G9" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="G9" s="10">
+      <c r="H9" s="10">
         <v>43</v>
       </c>
-      <c r="H9" s="10">
+      <c r="I9" s="10">
         <v>57.64</v>
       </c>
-      <c r="I9" s="10" t="s">
+      <c r="J9" s="10" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="10" spans="1:9">
-      <c r="A10" s="12" t="s">
+    <row r="10" spans="1:10">
+      <c r="A10" s="10">
+        <v>9</v>
+      </c>
+      <c r="B10" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="B10" s="12" t="s">
+      <c r="C10" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C10" s="12">
+      <c r="D10" s="12">
         <v>177</v>
       </c>
-      <c r="D10" s="13">
+      <c r="E10" s="13">
         <v>1.9305555555555555E-2</v>
       </c>
-      <c r="E10" s="12">
+      <c r="F10" s="12">
         <v>63</v>
       </c>
-      <c r="F10" s="12" t="s">
+      <c r="G10" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="G10" s="12">
+      <c r="H10" s="12">
         <v>42</v>
       </c>
-      <c r="H10" s="12">
+      <c r="I10" s="12">
         <v>50.68</v>
       </c>
-      <c r="I10" s="12" t="s">
+      <c r="J10" s="12" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="11" spans="1:9">
-      <c r="A11" s="12" t="s">
+    <row r="11" spans="1:10">
+      <c r="A11" s="10">
+        <v>10</v>
+      </c>
+      <c r="B11" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="B11" s="12" t="s">
+      <c r="C11" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C11" s="12">
+      <c r="D11" s="12">
         <v>99</v>
       </c>
-      <c r="D11" s="13">
+      <c r="E11" s="13">
         <v>9.7916666666666673E-3</v>
       </c>
-      <c r="E11" s="12">
+      <c r="F11" s="12">
         <v>63</v>
       </c>
-      <c r="F11" s="12" t="s">
+      <c r="G11" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="G11" s="12">
+      <c r="H11" s="12">
         <v>40</v>
       </c>
-      <c r="H11" s="12">
+      <c r="I11" s="12">
         <v>62.55</v>
       </c>
-      <c r="I11" s="12" t="s">
+      <c r="J11" s="12" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="12" spans="1:9">
-      <c r="A12" s="10" t="s">
+    <row r="12" spans="1:10">
+      <c r="A12" s="10">
+        <v>11</v>
+      </c>
+      <c r="B12" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="C12" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="C12" s="10">
+      <c r="D12" s="10">
         <v>185</v>
       </c>
-      <c r="D12" s="11">
+      <c r="E12" s="11">
         <v>1.6516203703703703E-2</v>
       </c>
-      <c r="E12" s="10">
+      <c r="F12" s="10">
         <v>63</v>
       </c>
-      <c r="F12" s="10" t="s">
+      <c r="G12" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="G12" s="10">
+      <c r="H12" s="10">
         <v>42</v>
       </c>
-      <c r="H12" s="10">
+      <c r="I12" s="10">
         <v>62.44</v>
       </c>
-      <c r="I12" s="10" t="s">
+      <c r="J12" s="10" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="13" spans="1:9">
-      <c r="A13" s="12" t="s">
+    <row r="13" spans="1:10">
+      <c r="A13" s="10">
+        <v>12</v>
+      </c>
+      <c r="B13" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="B13" s="12" t="s">
+      <c r="C13" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C13" s="12">
+      <c r="D13" s="12">
         <v>89</v>
       </c>
-      <c r="D13" s="13">
+      <c r="E13" s="13">
         <v>1.0532407407407407E-2</v>
       </c>
-      <c r="E13" s="12">
+      <c r="F13" s="12">
         <v>63</v>
       </c>
-      <c r="F13" s="12" t="s">
+      <c r="G13" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="G13" s="12">
+      <c r="H13" s="12">
         <v>34</v>
       </c>
-      <c r="H13" s="12">
+      <c r="I13" s="12">
         <v>58.09</v>
       </c>
-      <c r="I13" s="12" t="s">
+      <c r="J13" s="12" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="14" spans="1:9">
-      <c r="A14" s="10" t="s">
+    <row r="14" spans="1:10">
+      <c r="A14" s="10">
+        <v>13</v>
+      </c>
+      <c r="B14" s="10" t="s">
         <v>94</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="C14" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="C14" s="10">
+      <c r="D14" s="10">
         <v>167</v>
       </c>
-      <c r="D14" s="11">
+      <c r="E14" s="11">
         <v>1.9953703703703703E-2</v>
       </c>
-      <c r="E14" s="10">
+      <c r="F14" s="10">
         <v>55</v>
       </c>
-      <c r="F14" s="10" t="s">
+      <c r="G14" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="G14" s="10">
+      <c r="H14" s="10">
         <v>39</v>
       </c>
-      <c r="H14" s="10">
+      <c r="I14" s="10">
         <v>53.35</v>
       </c>
-      <c r="I14" s="10" t="s">
+      <c r="J14" s="10" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="15" spans="1:9">
-      <c r="A15" s="10" t="s">
+    <row r="15" spans="1:10">
+      <c r="A15" s="10">
+        <v>14</v>
+      </c>
+      <c r="B15" s="10" t="s">
         <v>97</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="C15" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="C15" s="10">
+      <c r="D15" s="10">
         <v>122</v>
       </c>
-      <c r="D15" s="11">
+      <c r="E15" s="11">
         <v>1.1215277777777777E-2</v>
       </c>
-      <c r="E15" s="10">
+      <c r="F15" s="10">
         <v>63</v>
       </c>
-      <c r="F15" s="10" t="s">
+      <c r="G15" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="G15" s="10">
+      <c r="H15" s="10">
         <v>43</v>
       </c>
-      <c r="H15" s="10">
+      <c r="I15" s="10">
         <v>65.33</v>
       </c>
-      <c r="I15" s="10" t="s">
+      <c r="J15" s="10" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="16" spans="1:9">
-      <c r="A16" s="12" t="s">
+    <row r="16" spans="1:10">
+      <c r="A16" s="10">
+        <v>15</v>
+      </c>
+      <c r="B16" s="12" t="s">
         <v>99</v>
       </c>
-      <c r="B16" s="12" t="s">
+      <c r="C16" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C16" s="12">
+      <c r="D16" s="12">
         <v>117</v>
       </c>
-      <c r="D16" s="13">
+      <c r="E16" s="13">
         <v>1.1168981481481481E-2</v>
       </c>
-      <c r="E16" s="12">
+      <c r="F16" s="12">
         <v>63</v>
       </c>
-      <c r="F16" s="12" t="s">
+      <c r="G16" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="G16" s="12">
+      <c r="H16" s="12">
         <v>38</v>
       </c>
-      <c r="H16" s="12">
+      <c r="I16" s="12">
         <v>60.5</v>
       </c>
-      <c r="I16" s="12" t="s">
+      <c r="J16" s="12" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="17" spans="1:10">
-      <c r="A17" s="10" t="s">
+    <row r="17" spans="1:11">
+      <c r="A17" s="10">
+        <v>16</v>
+      </c>
+      <c r="B17" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="B17" s="10" t="s">
+      <c r="C17" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="C17" s="10">
+      <c r="D17" s="10">
         <v>171</v>
       </c>
-      <c r="D17" s="11">
+      <c r="E17" s="11">
         <v>1.3865740740740741E-2</v>
       </c>
-      <c r="E17" s="10">
+      <c r="F17" s="10">
         <v>63</v>
       </c>
-      <c r="F17" s="10" t="s">
+      <c r="G17" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="G17" s="10">
+      <c r="H17" s="10">
         <v>43</v>
       </c>
-      <c r="H17" s="10">
+      <c r="I17" s="10">
         <v>58</v>
       </c>
-      <c r="I17" s="10" t="s">
+      <c r="J17" s="10" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="18" spans="1:10">
-      <c r="A18" s="12" t="s">
+    <row r="18" spans="1:11">
+      <c r="A18" s="10">
+        <v>17</v>
+      </c>
+      <c r="B18" s="12" t="s">
         <v>103</v>
       </c>
-      <c r="B18" s="12" t="s">
+      <c r="C18" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C18" s="12">
+      <c r="D18" s="12">
         <v>258</v>
       </c>
-      <c r="D18" s="13">
+      <c r="E18" s="13">
         <v>1.892361111111111E-2</v>
       </c>
-      <c r="E18" s="12">
+      <c r="F18" s="12">
         <v>55</v>
       </c>
-      <c r="F18" s="12" t="s">
+      <c r="G18" s="12" t="s">
         <v>95</v>
       </c>
-      <c r="G18" s="12">
+      <c r="H18" s="12">
         <v>37</v>
       </c>
-      <c r="H18" s="12">
+      <c r="I18" s="12">
         <v>55.12</v>
       </c>
-      <c r="I18" s="12" t="s">
+      <c r="J18" s="12" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="19" spans="1:10">
-      <c r="A19" s="14" t="s">
+    <row r="19" spans="1:11">
+      <c r="A19" s="14"/>
+      <c r="B19" s="14" t="s">
         <v>105</v>
       </c>
-      <c r="B19" s="14" t="s">
+      <c r="C19" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="C19" s="14">
+      <c r="D19" s="14">
         <v>216</v>
       </c>
-      <c r="D19" s="15">
+      <c r="E19" s="15">
         <v>1.8599537037037036E-2</v>
       </c>
-      <c r="E19" s="14">
+      <c r="F19" s="14">
         <v>63</v>
       </c>
-      <c r="F19" s="14" t="s">
+      <c r="G19" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="G19" s="14">
+      <c r="H19" s="14">
         <v>39</v>
       </c>
-      <c r="H19" s="14">
+      <c r="I19" s="14">
         <v>46.93</v>
       </c>
-      <c r="I19" s="14" t="s">
+      <c r="J19" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="J19" s="27" t="s">
+      <c r="K19" s="27" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="20" spans="1:10">
-      <c r="A20" s="12" t="s">
+    <row r="20" spans="1:11">
+      <c r="A20" s="12">
+        <v>18</v>
+      </c>
+      <c r="B20" s="12" t="s">
         <v>107</v>
       </c>
-      <c r="B20" s="12" t="s">
+      <c r="C20" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C20" s="12">
+      <c r="D20" s="12">
         <v>93</v>
       </c>
-      <c r="D20" s="13">
+      <c r="E20" s="13">
         <v>9.3981481481481485E-3</v>
       </c>
-      <c r="E20" s="12">
+      <c r="F20" s="12">
         <v>63</v>
       </c>
-      <c r="F20" s="12" t="s">
+      <c r="G20" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="G20" s="12">
+      <c r="H20" s="12">
         <v>41</v>
       </c>
-      <c r="H20" s="12">
+      <c r="I20" s="12">
         <v>64.36</v>
       </c>
-      <c r="I20" s="12" t="s">
+      <c r="J20" s="12" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="21" spans="1:10">
-      <c r="A21" s="12" t="s">
+    <row r="21" spans="1:11">
+      <c r="A21" s="12">
+        <v>19</v>
+      </c>
+      <c r="B21" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="B21" s="12" t="s">
+      <c r="C21" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C21" s="12">
+      <c r="D21" s="12">
         <v>172</v>
       </c>
-      <c r="D21" s="13">
+      <c r="E21" s="13">
         <v>1.5462962962962963E-2</v>
       </c>
-      <c r="E21" s="12">
+      <c r="F21" s="12">
         <v>63</v>
       </c>
-      <c r="F21" s="12" t="s">
+      <c r="G21" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="G21" s="12">
+      <c r="H21" s="12">
         <v>39</v>
       </c>
-      <c r="H21" s="12">
+      <c r="I21" s="12">
         <v>74.459999999999994</v>
       </c>
-      <c r="I21" s="12" t="s">
+      <c r="J21" s="12" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="22" spans="1:10">
-      <c r="A22" s="10" t="s">
+    <row r="22" spans="1:11">
+      <c r="A22" s="12">
+        <v>20</v>
+      </c>
+      <c r="B22" s="10" t="s">
         <v>111</v>
       </c>
-      <c r="B22" s="10" t="s">
+      <c r="C22" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="C22" s="10">
+      <c r="D22" s="10">
         <v>125</v>
       </c>
-      <c r="D22" s="11">
+      <c r="E22" s="11">
         <v>8.6805555555555559E-3</v>
       </c>
-      <c r="E22" s="10">
+      <c r="F22" s="10">
         <v>63</v>
       </c>
-      <c r="F22" s="10" t="s">
+      <c r="G22" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="G22" s="10">
+      <c r="H22" s="10">
         <v>42</v>
       </c>
-      <c r="H22" s="10">
+      <c r="I22" s="10">
         <v>70.56</v>
       </c>
-      <c r="I22" s="10" t="s">
+      <c r="J22" s="10" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="23" spans="1:10">
-      <c r="A23" s="12" t="s">
+    <row r="23" spans="1:11">
+      <c r="A23" s="12">
+        <v>21</v>
+      </c>
+      <c r="B23" s="12" t="s">
         <v>113</v>
       </c>
-      <c r="B23" s="12" t="s">
+      <c r="C23" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C23" s="12">
+      <c r="D23" s="12">
         <v>189</v>
       </c>
-      <c r="D23" s="13">
+      <c r="E23" s="13">
         <v>1.4305555555555556E-2</v>
       </c>
-      <c r="E23" s="12">
+      <c r="F23" s="12">
         <v>63</v>
       </c>
-      <c r="F23" s="12" t="s">
+      <c r="G23" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="G23" s="12">
+      <c r="H23" s="12">
         <v>41</v>
       </c>
-      <c r="H23" s="12">
+      <c r="I23" s="12">
         <v>76.8</v>
       </c>
-      <c r="I23" s="12" t="s">
+      <c r="J23" s="12" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="24" spans="1:10">
-      <c r="A24" s="12" t="s">
+    <row r="24" spans="1:11">
+      <c r="A24" s="12">
+        <v>22</v>
+      </c>
+      <c r="B24" s="12" t="s">
         <v>115</v>
       </c>
-      <c r="B24" s="12" t="s">
+      <c r="C24" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C24" s="12">
+      <c r="D24" s="12">
         <v>422</v>
       </c>
-      <c r="D24" s="13">
+      <c r="E24" s="13">
         <v>3.1041666666666665E-2</v>
       </c>
-      <c r="E24" s="12">
+      <c r="F24" s="12">
         <v>63</v>
       </c>
-      <c r="F24" s="12" t="s">
+      <c r="G24" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="G24" s="12">
+      <c r="H24" s="12">
         <v>42</v>
       </c>
-      <c r="H24" s="12">
+      <c r="I24" s="12">
         <v>53.02</v>
       </c>
-      <c r="I24" s="12" t="s">
+      <c r="J24" s="12" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="25" spans="1:10">
-      <c r="A25" s="12" t="s">
+    <row r="25" spans="1:11">
+      <c r="A25" s="12">
+        <v>23</v>
+      </c>
+      <c r="B25" s="12" t="s">
         <v>117</v>
       </c>
-      <c r="B25" s="12" t="s">
+      <c r="C25" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C25" s="12">
+      <c r="D25" s="12">
         <v>192</v>
       </c>
-      <c r="D25" s="13">
+      <c r="E25" s="13">
         <v>1.3796296296296296E-2</v>
       </c>
-      <c r="E25" s="12">
+      <c r="F25" s="12">
         <v>63</v>
       </c>
-      <c r="F25" s="12" t="s">
+      <c r="G25" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="G25" s="12">
+      <c r="H25" s="12">
         <v>36</v>
       </c>
-      <c r="H25" s="12">
+      <c r="I25" s="12">
         <v>69.510000000000005</v>
       </c>
-      <c r="I25" s="12" t="s">
+      <c r="J25" s="12" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="26" spans="1:10">
-      <c r="A26" s="10" t="s">
+    <row r="26" spans="1:11">
+      <c r="A26" s="12">
+        <v>24</v>
+      </c>
+      <c r="B26" s="10" t="s">
         <v>119</v>
       </c>
-      <c r="B26" s="10" t="s">
+      <c r="C26" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="C26" s="10">
+      <c r="D26" s="10">
         <v>125</v>
       </c>
-      <c r="D26" s="11">
+      <c r="E26" s="11">
         <v>1.1747685185185186E-2</v>
       </c>
-      <c r="E26" s="10">
+      <c r="F26" s="10">
         <v>63</v>
       </c>
-      <c r="F26" s="10" t="s">
+      <c r="G26" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="G26" s="10">
+      <c r="H26" s="10">
         <v>42</v>
       </c>
-      <c r="H26" s="10">
+      <c r="I26" s="10">
         <v>60.41</v>
       </c>
-      <c r="I26" s="10" t="s">
+      <c r="J26" s="10" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="27" spans="1:10">
-      <c r="A27" s="12" t="s">
+    <row r="27" spans="1:11">
+      <c r="A27" s="12">
+        <v>25</v>
+      </c>
+      <c r="B27" s="12" t="s">
         <v>121</v>
       </c>
-      <c r="B27" s="12" t="s">
+      <c r="C27" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C27" s="12">
+      <c r="D27" s="12">
         <v>153</v>
       </c>
-      <c r="D27" s="13">
+      <c r="E27" s="13">
         <v>1.457175925925926E-2</v>
       </c>
-      <c r="E27" s="12">
+      <c r="F27" s="12">
         <v>63</v>
       </c>
-      <c r="F27" s="12" t="s">
+      <c r="G27" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="G27" s="12">
+      <c r="H27" s="12">
         <v>32</v>
       </c>
-      <c r="H27" s="12">
+      <c r="I27" s="12">
         <v>66.39</v>
       </c>
-      <c r="I27" s="12" t="s">
+      <c r="J27" s="12" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="28" spans="1:10">
-      <c r="A28" s="10" t="s">
+    <row r="28" spans="1:11">
+      <c r="A28" s="12">
+        <v>26</v>
+      </c>
+      <c r="B28" s="10" t="s">
         <v>123</v>
       </c>
-      <c r="B28" s="10" t="s">
+      <c r="C28" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="C28" s="10">
+      <c r="D28" s="10">
         <v>217</v>
       </c>
-      <c r="D28" s="11">
+      <c r="E28" s="11">
         <v>1.4849537037037038E-2</v>
       </c>
-      <c r="E28" s="10">
+      <c r="F28" s="10">
         <v>63</v>
       </c>
-      <c r="F28" s="10" t="s">
+      <c r="G28" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="G28" s="10">
+      <c r="H28" s="10">
         <v>43</v>
       </c>
-      <c r="H28" s="10">
+      <c r="I28" s="10">
         <v>54.72</v>
       </c>
-      <c r="I28" s="10" t="s">
+      <c r="J28" s="10" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="29" spans="1:10">
-      <c r="A29" s="10" t="s">
+    <row r="29" spans="1:11">
+      <c r="A29" s="12">
+        <v>27</v>
+      </c>
+      <c r="B29" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="B29" s="10" t="s">
+      <c r="C29" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="C29" s="10">
+      <c r="D29" s="10">
         <v>163</v>
       </c>
-      <c r="D29" s="11">
+      <c r="E29" s="11">
         <v>1.3460648148148149E-2</v>
       </c>
-      <c r="E29" s="10">
+      <c r="F29" s="10">
         <v>63</v>
       </c>
-      <c r="F29" s="10" t="s">
+      <c r="G29" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="G29" s="10">
+      <c r="H29" s="10">
         <v>42</v>
       </c>
-      <c r="H29" s="10">
+      <c r="I29" s="10">
         <v>56.7</v>
       </c>
-      <c r="I29" s="10" t="s">
+      <c r="J29" s="10" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="30" spans="1:10">
-      <c r="A30" s="12" t="s">
+    <row r="30" spans="1:11">
+      <c r="A30" s="12">
+        <v>28</v>
+      </c>
+      <c r="B30" s="12" t="s">
         <v>127</v>
       </c>
-      <c r="B30" s="12" t="s">
+      <c r="C30" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C30" s="12">
+      <c r="D30" s="12">
         <v>140</v>
       </c>
-      <c r="D30" s="13">
+      <c r="E30" s="13">
         <v>1.1817129629629629E-2</v>
       </c>
-      <c r="E30" s="12">
+      <c r="F30" s="12">
         <v>63</v>
       </c>
-      <c r="F30" s="12" t="s">
+      <c r="G30" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="G30" s="12">
+      <c r="H30" s="12">
         <v>34</v>
       </c>
-      <c r="H30" s="12">
+      <c r="I30" s="12">
         <v>61.47</v>
       </c>
-      <c r="I30" s="12" t="s">
+      <c r="J30" s="12" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="31" spans="1:10">
-      <c r="A31" s="10" t="s">
+    <row r="31" spans="1:11">
+      <c r="A31" s="12">
+        <v>29</v>
+      </c>
+      <c r="B31" s="10" t="s">
         <v>129</v>
       </c>
-      <c r="B31" s="10" t="s">
+      <c r="C31" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="C31" s="10">
+      <c r="D31" s="10">
         <v>200</v>
       </c>
-      <c r="D31" s="11">
+      <c r="E31" s="11">
         <v>1.8668981481481481E-2</v>
       </c>
-      <c r="E31" s="10">
+      <c r="F31" s="10">
         <v>63</v>
       </c>
-      <c r="F31" s="10" t="s">
+      <c r="G31" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="G31" s="10">
+      <c r="H31" s="10">
         <v>43</v>
       </c>
-      <c r="H31" s="10">
+      <c r="I31" s="10">
         <v>54.23</v>
       </c>
-      <c r="I31" s="10" t="s">
+      <c r="J31" s="10" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="32" spans="1:10">
-      <c r="A32" s="14" t="s">
+    <row r="32" spans="1:11">
+      <c r="A32" s="14"/>
+      <c r="B32" s="14" t="s">
         <v>131</v>
       </c>
-      <c r="B32" s="14" t="s">
+      <c r="C32" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="C32" s="14">
+      <c r="D32" s="14">
         <v>57</v>
       </c>
-      <c r="D32" s="15">
+      <c r="E32" s="15">
         <v>8.9120370370370378E-3</v>
       </c>
-      <c r="E32" s="14">
+      <c r="F32" s="14">
         <v>63</v>
       </c>
-      <c r="F32" s="14" t="s">
+      <c r="G32" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="G32" s="14">
+      <c r="H32" s="14">
         <v>43</v>
       </c>
-      <c r="H32" s="14">
+      <c r="I32" s="14">
         <v>62.88</v>
       </c>
-      <c r="I32" s="14" t="s">
+      <c r="J32" s="14" t="s">
         <v>132</v>
       </c>
-      <c r="J32" s="27" t="s">
+      <c r="K32" s="27" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="33" spans="1:9">
-      <c r="A33" s="12" t="s">
+    <row r="33" spans="1:10">
+      <c r="A33" s="12">
+        <v>30</v>
+      </c>
+      <c r="B33" s="12" t="s">
         <v>133</v>
       </c>
-      <c r="B33" s="12" t="s">
+      <c r="C33" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C33" s="12">
+      <c r="D33" s="12">
         <v>63</v>
       </c>
-      <c r="D33" s="13">
+      <c r="E33" s="13">
         <v>7.5231481481481477E-3</v>
       </c>
-      <c r="E33" s="12">
+      <c r="F33" s="12">
         <v>63</v>
       </c>
-      <c r="F33" s="12" t="s">
+      <c r="G33" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="G33" s="12">
+      <c r="H33" s="12">
         <v>30</v>
       </c>
-      <c r="H33" s="12">
+      <c r="I33" s="12">
         <v>75.319999999999993</v>
       </c>
-      <c r="I33" s="12" t="s">
+      <c r="J33" s="12" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="34" spans="1:9">
-      <c r="A34" s="10" t="s">
+    <row r="34" spans="1:10">
+      <c r="A34" s="10">
+        <v>31</v>
+      </c>
+      <c r="B34" s="10" t="s">
         <v>135</v>
       </c>
-      <c r="B34" s="10" t="s">
+      <c r="C34" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="C34" s="10">
+      <c r="D34" s="10">
         <v>114</v>
       </c>
-      <c r="D34" s="11">
+      <c r="E34" s="11">
         <v>1.1122685185185185E-2</v>
       </c>
-      <c r="E34" s="10">
+      <c r="F34" s="10">
         <v>63</v>
       </c>
-      <c r="F34" s="10" t="s">
+      <c r="G34" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="G34" s="10">
+      <c r="H34" s="10">
         <v>42</v>
       </c>
-      <c r="H34" s="10">
+      <c r="I34" s="10">
         <v>62.31</v>
       </c>
-      <c r="I34" s="10" t="s">
+      <c r="J34" s="10" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="35" spans="1:9">
-      <c r="A35" s="12" t="s">
+    <row r="35" spans="1:10">
+      <c r="A35" s="12">
+        <v>32</v>
+      </c>
+      <c r="B35" s="12" t="s">
         <v>137</v>
       </c>
-      <c r="B35" s="12" t="s">
+      <c r="C35" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C35" s="12">
+      <c r="D35" s="12">
         <v>530</v>
       </c>
-      <c r="D35" s="13">
+      <c r="E35" s="13">
         <v>3.5960648148148151E-2</v>
       </c>
-      <c r="E35" s="12">
+      <c r="F35" s="12">
         <v>63</v>
       </c>
-      <c r="F35" s="12" t="s">
+      <c r="G35" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="G35" s="12">
+      <c r="H35" s="12">
         <v>37</v>
       </c>
-      <c r="H35" s="12">
+      <c r="I35" s="12">
         <v>57.9</v>
       </c>
-      <c r="I35" s="12" t="s">
+      <c r="J35" s="12" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="36" spans="1:9">
-      <c r="A36" s="10" t="s">
+    <row r="36" spans="1:10">
+      <c r="A36" s="10">
+        <v>33</v>
+      </c>
+      <c r="B36" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="B36" s="10" t="s">
+      <c r="C36" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="C36" s="10">
+      <c r="D36" s="10">
         <v>126</v>
       </c>
-      <c r="D36" s="11">
+      <c r="E36" s="11">
         <v>9.9305555555555553E-3</v>
       </c>
-      <c r="E36" s="10">
+      <c r="F36" s="10">
         <v>63</v>
       </c>
-      <c r="F36" s="10" t="s">
+      <c r="G36" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="G36" s="10">
+      <c r="H36" s="10">
         <v>41</v>
       </c>
-      <c r="H36" s="10">
+      <c r="I36" s="10">
         <v>74.83</v>
       </c>
-      <c r="I36" s="10" t="s">
+      <c r="J36" s="10" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="37" spans="1:9">
-      <c r="A37" s="10" t="s">
+    <row r="37" spans="1:10">
+      <c r="A37" s="12">
+        <v>34</v>
+      </c>
+      <c r="B37" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="B37" s="10" t="s">
+      <c r="C37" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="C37" s="10">
+      <c r="D37" s="10">
         <v>116</v>
       </c>
-      <c r="D37" s="11">
+      <c r="E37" s="11">
         <v>9.2592592592592587E-3</v>
       </c>
-      <c r="E37" s="10">
+      <c r="F37" s="10">
         <v>63</v>
       </c>
-      <c r="F37" s="10" t="s">
+      <c r="G37" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="G37" s="10">
+      <c r="H37" s="10">
         <v>41</v>
       </c>
-      <c r="H37" s="10">
+      <c r="I37" s="10">
         <v>81.900000000000006</v>
       </c>
-      <c r="I37" s="10" t="s">
+      <c r="J37" s="10" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="38" spans="1:9">
-      <c r="A38" s="12" t="s">
+    <row r="38" spans="1:10">
+      <c r="A38" s="10">
+        <v>35</v>
+      </c>
+      <c r="B38" s="12" t="s">
         <v>143</v>
       </c>
-      <c r="B38" s="12" t="s">
+      <c r="C38" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C38" s="12">
+      <c r="D38" s="12">
         <v>71</v>
       </c>
-      <c r="D38" s="13">
+      <c r="E38" s="13">
         <v>8.8078703703703704E-3</v>
       </c>
-      <c r="E38" s="12">
+      <c r="F38" s="12">
         <v>63</v>
       </c>
-      <c r="F38" s="12" t="s">
+      <c r="G38" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="G38" s="12">
+      <c r="H38" s="12">
         <v>37</v>
       </c>
-      <c r="H38" s="12">
+      <c r="I38" s="12">
         <v>71.91</v>
       </c>
-      <c r="I38" s="12" t="s">
+      <c r="J38" s="12" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="39" spans="1:9">
-      <c r="A39" s="10" t="s">
+    <row r="39" spans="1:10">
+      <c r="A39" s="12">
+        <v>36</v>
+      </c>
+      <c r="B39" s="10" t="s">
         <v>145</v>
       </c>
-      <c r="B39" s="10" t="s">
+      <c r="C39" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="C39" s="10">
+      <c r="D39" s="10">
         <v>61</v>
       </c>
-      <c r="D39" s="11">
+      <c r="E39" s="11">
         <v>9.3634259259259261E-3</v>
       </c>
-      <c r="E39" s="10">
+      <c r="F39" s="10">
         <v>63</v>
       </c>
-      <c r="F39" s="10" t="s">
+      <c r="G39" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="G39" s="10">
+      <c r="H39" s="10">
         <v>43</v>
       </c>
-      <c r="H39" s="10">
+      <c r="I39" s="10">
         <v>55.25</v>
       </c>
-      <c r="I39" s="10" t="s">
+      <c r="J39" s="10" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="40" spans="1:9">
-      <c r="A40" s="12" t="s">
+    <row r="40" spans="1:10">
+      <c r="A40" s="10">
+        <v>37</v>
+      </c>
+      <c r="B40" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="B40" s="12" t="s">
+      <c r="C40" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C40" s="12">
+      <c r="D40" s="12">
         <v>142</v>
       </c>
-      <c r="D40" s="13">
+      <c r="E40" s="13">
         <v>1.7696759259259259E-2</v>
       </c>
-      <c r="E40" s="12">
+      <c r="F40" s="12">
         <v>63</v>
       </c>
-      <c r="F40" s="12" t="s">
+      <c r="G40" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="G40" s="12">
+      <c r="H40" s="12">
         <v>41</v>
       </c>
-      <c r="H40" s="12">
+      <c r="I40" s="12">
         <v>43.09</v>
       </c>
-      <c r="I40" s="12" t="s">
+      <c r="J40" s="12" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="41" spans="1:9">
-      <c r="A41" s="10" t="s">
+    <row r="41" spans="1:10">
+      <c r="A41" s="12">
+        <v>38</v>
+      </c>
+      <c r="B41" s="10" t="s">
         <v>149</v>
       </c>
-      <c r="B41" s="10" t="s">
+      <c r="C41" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="C41" s="10">
+      <c r="D41" s="10">
         <v>264</v>
       </c>
-      <c r="D41" s="11">
+      <c r="E41" s="11">
         <v>2.0416666666666666E-2</v>
       </c>
-      <c r="E41" s="10">
+      <c r="F41" s="10">
         <v>63</v>
       </c>
-      <c r="F41" s="10" t="s">
+      <c r="G41" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="G41" s="10">
+      <c r="H41" s="10">
         <v>43</v>
       </c>
-      <c r="H41" s="10">
+      <c r="I41" s="10">
         <v>54.12</v>
       </c>
-      <c r="I41" s="10" t="s">
+      <c r="J41" s="10" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="42" spans="1:9">
-      <c r="A42" s="12" t="s">
+    <row r="42" spans="1:10">
+      <c r="A42" s="10">
+        <v>39</v>
+      </c>
+      <c r="B42" s="12" t="s">
         <v>151</v>
       </c>
-      <c r="B42" s="12" t="s">
+      <c r="C42" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C42" s="12">
+      <c r="D42" s="12">
         <v>100</v>
       </c>
-      <c r="D42" s="13">
+      <c r="E42" s="13">
         <v>1.1550925925925926E-2</v>
       </c>
-      <c r="E42" s="12">
+      <c r="F42" s="12">
         <v>63</v>
       </c>
-      <c r="F42" s="12" t="s">
+      <c r="G42" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="G42" s="12">
+      <c r="H42" s="12">
         <v>32</v>
       </c>
-      <c r="H42" s="12">
+      <c r="I42" s="12">
         <v>66.31</v>
       </c>
-      <c r="I42" s="12" t="s">
+      <c r="J42" s="12" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="43" spans="1:9">
-      <c r="A43" s="10" t="s">
+    <row r="43" spans="1:10">
+      <c r="A43" s="12">
+        <v>40</v>
+      </c>
+      <c r="B43" s="10" t="s">
         <v>153</v>
       </c>
-      <c r="B43" s="10" t="s">
+      <c r="C43" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="C43" s="10">
+      <c r="D43" s="10">
         <v>93</v>
       </c>
-      <c r="D43" s="11">
+      <c r="E43" s="11">
         <v>9.432870370370371E-3</v>
       </c>
-      <c r="E43" s="10">
+      <c r="F43" s="10">
         <v>63</v>
       </c>
-      <c r="F43" s="10" t="s">
+      <c r="G43" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="G43" s="10">
+      <c r="H43" s="10">
         <v>43</v>
       </c>
-      <c r="H43" s="10">
+      <c r="I43" s="10">
         <v>62.5</v>
       </c>
-      <c r="I43" s="10" t="s">
+      <c r="J43" s="10" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="44" spans="1:9">
-      <c r="A44" s="12" t="s">
+    <row r="44" spans="1:10">
+      <c r="A44" s="10">
+        <v>41</v>
+      </c>
+      <c r="B44" s="12" t="s">
         <v>155</v>
       </c>
-      <c r="B44" s="12" t="s">
+      <c r="C44" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C44" s="12">
+      <c r="D44" s="12">
         <v>81</v>
       </c>
-      <c r="D44" s="13">
+      <c r="E44" s="13">
         <v>8.8310185185185193E-3</v>
       </c>
-      <c r="E44" s="12">
+      <c r="F44" s="12">
         <v>63</v>
       </c>
-      <c r="F44" s="12" t="s">
+      <c r="G44" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="G44" s="12">
+      <c r="H44" s="12">
         <v>31</v>
       </c>
-      <c r="H44" s="12">
+      <c r="I44" s="12">
         <v>55.05</v>
       </c>
-      <c r="I44" s="12" t="s">
+      <c r="J44" s="12" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="45" spans="1:9">
-      <c r="A45" s="10" t="s">
+    <row r="45" spans="1:10">
+      <c r="A45" s="12">
+        <v>42</v>
+      </c>
+      <c r="B45" s="10" t="s">
         <v>157</v>
       </c>
-      <c r="B45" s="10" t="s">
+      <c r="C45" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="C45" s="10">
+      <c r="D45" s="10">
         <v>109</v>
       </c>
-      <c r="D45" s="11">
+      <c r="E45" s="11">
         <v>1.0717592592592593E-2</v>
       </c>
-      <c r="E45" s="10">
+      <c r="F45" s="10">
         <v>63</v>
       </c>
-      <c r="F45" s="10" t="s">
+      <c r="G45" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="G45" s="10">
+      <c r="H45" s="10">
         <v>40</v>
       </c>
-      <c r="H45" s="10">
+      <c r="I45" s="10">
         <v>53.65</v>
       </c>
-      <c r="I45" s="10" t="s">
+      <c r="J45" s="10" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="46" spans="1:9">
-      <c r="A46" s="12" t="s">
+    <row r="46" spans="1:10">
+      <c r="A46" s="10">
+        <v>43</v>
+      </c>
+      <c r="B46" s="12" t="s">
         <v>159</v>
       </c>
-      <c r="B46" s="12" t="s">
+      <c r="C46" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C46" s="12">
+      <c r="D46" s="12">
         <v>405</v>
       </c>
-      <c r="D46" s="13">
+      <c r="E46" s="13">
         <v>2.8506944444444446E-2</v>
       </c>
-      <c r="E46" s="12">
+      <c r="F46" s="12">
         <v>63</v>
       </c>
-      <c r="F46" s="12" t="s">
+      <c r="G46" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="G46" s="12">
+      <c r="H46" s="12">
         <v>42</v>
       </c>
-      <c r="H46" s="12">
+      <c r="I46" s="12">
         <v>45.94</v>
       </c>
-      <c r="I46" s="12" t="s">
+      <c r="J46" s="12" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="47" spans="1:9">
-      <c r="A47" s="10" t="s">
+    <row r="47" spans="1:10">
+      <c r="A47" s="12">
+        <v>44</v>
+      </c>
+      <c r="B47" s="10" t="s">
         <v>161</v>
       </c>
-      <c r="B47" s="10" t="s">
+      <c r="C47" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="C47" s="10">
+      <c r="D47" s="10">
         <v>113</v>
       </c>
-      <c r="D47" s="11">
+      <c r="E47" s="11">
         <v>1.0104166666666666E-2</v>
       </c>
-      <c r="E47" s="10">
+      <c r="F47" s="10">
         <v>63</v>
       </c>
-      <c r="F47" s="10" t="s">
+      <c r="G47" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="G47" s="10">
+      <c r="H47" s="10">
         <v>43</v>
       </c>
-      <c r="H47" s="10">
+      <c r="I47" s="10">
         <v>60.14</v>
       </c>
-      <c r="I47" s="10" t="s">
+      <c r="J47" s="10" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="48" spans="1:9">
-      <c r="A48" s="12" t="s">
+    <row r="48" spans="1:10">
+      <c r="A48" s="10">
+        <v>45</v>
+      </c>
+      <c r="B48" s="12" t="s">
         <v>163</v>
       </c>
-      <c r="B48" s="12" t="s">
+      <c r="C48" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C48" s="12">
+      <c r="D48" s="12">
         <v>289</v>
       </c>
-      <c r="D48" s="13">
+      <c r="E48" s="13">
         <v>2.1087962962962965E-2</v>
       </c>
-      <c r="E48" s="12">
+      <c r="F48" s="12">
         <v>63</v>
       </c>
-      <c r="F48" s="12" t="s">
+      <c r="G48" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="G48" s="12">
+      <c r="H48" s="12">
         <v>37</v>
       </c>
-      <c r="H48" s="12">
+      <c r="I48" s="12">
         <v>66.819999999999993</v>
       </c>
-      <c r="I48" s="12" t="s">
+      <c r="J48" s="12" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="49" spans="1:9">
-      <c r="A49" s="12" t="s">
+    <row r="49" spans="1:10">
+      <c r="A49" s="12">
+        <v>46</v>
+      </c>
+      <c r="B49" s="12" t="s">
         <v>165</v>
       </c>
-      <c r="B49" s="12" t="s">
+      <c r="C49" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C49" s="12">
+      <c r="D49" s="12">
         <v>132</v>
       </c>
-      <c r="D49" s="13">
+      <c r="E49" s="13">
         <v>1.1828703703703704E-2</v>
       </c>
-      <c r="E49" s="12">
+      <c r="F49" s="12">
         <v>63</v>
       </c>
-      <c r="F49" s="12" t="s">
+      <c r="G49" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="G49" s="12">
+      <c r="H49" s="12">
         <v>34</v>
       </c>
-      <c r="H49" s="12">
+      <c r="I49" s="12">
         <v>53.37</v>
       </c>
-      <c r="I49" s="12" t="s">
+      <c r="J49" s="12" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="50" spans="1:9">
-      <c r="A50" s="10" t="s">
+    <row r="50" spans="1:10">
+      <c r="A50" s="10">
+        <v>47</v>
+      </c>
+      <c r="B50" s="10" t="s">
         <v>167</v>
       </c>
-      <c r="B50" s="10" t="s">
+      <c r="C50" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="C50" s="10">
+      <c r="D50" s="10">
         <v>122</v>
       </c>
-      <c r="D50" s="11">
+      <c r="E50" s="11">
         <v>1.005787037037037E-2</v>
       </c>
-      <c r="E50" s="10">
+      <c r="F50" s="10">
         <v>63</v>
       </c>
-      <c r="F50" s="10" t="s">
+      <c r="G50" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="G50" s="10">
+      <c r="H50" s="10">
         <v>43</v>
       </c>
-      <c r="H50" s="10">
+      <c r="I50" s="10">
         <v>64.7</v>
       </c>
-      <c r="I50" s="10" t="s">
+      <c r="J50" s="10" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="51" spans="1:9">
-      <c r="A51" s="12" t="s">
+    <row r="51" spans="1:10">
+      <c r="A51" s="12">
+        <v>48</v>
+      </c>
+      <c r="B51" s="12" t="s">
         <v>169</v>
       </c>
-      <c r="B51" s="12" t="s">
+      <c r="C51" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C51" s="12">
+      <c r="D51" s="12">
         <v>371</v>
       </c>
-      <c r="D51" s="13">
+      <c r="E51" s="13">
         <v>2.78125E-2</v>
       </c>
-      <c r="E51" s="12">
+      <c r="F51" s="12">
         <v>63</v>
       </c>
-      <c r="F51" s="12" t="s">
+      <c r="G51" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="G51" s="12">
+      <c r="H51" s="12">
         <v>41</v>
       </c>
-      <c r="H51" s="12">
+      <c r="I51" s="12">
         <v>47.72</v>
       </c>
-      <c r="I51" s="12" t="s">
+      <c r="J51" s="12" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="52" spans="1:9">
-      <c r="A52" s="10" t="s">
+    <row r="52" spans="1:10">
+      <c r="A52" s="10">
+        <v>49</v>
+      </c>
+      <c r="B52" s="10" t="s">
         <v>171</v>
       </c>
-      <c r="B52" s="10" t="s">
+      <c r="C52" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="C52" s="10">
+      <c r="D52" s="10">
         <v>134</v>
       </c>
-      <c r="D52" s="11">
+      <c r="E52" s="11">
         <v>1.1770833333333333E-2</v>
       </c>
-      <c r="E52" s="10">
+      <c r="F52" s="10">
         <v>63</v>
       </c>
-      <c r="F52" s="10" t="s">
+      <c r="G52" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="G52" s="10">
+      <c r="H52" s="10">
         <v>41</v>
       </c>
-      <c r="H52" s="10">
+      <c r="I52" s="10">
         <v>60.88</v>
       </c>
-      <c r="I52" s="10" t="s">
+      <c r="J52" s="10" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="53" spans="1:9">
-      <c r="A53" s="10" t="s">
+    <row r="53" spans="1:10">
+      <c r="A53" s="12">
+        <v>50</v>
+      </c>
+      <c r="B53" s="10" t="s">
         <v>173</v>
       </c>
-      <c r="B53" s="10" t="s">
+      <c r="C53" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="C53" s="10">
+      <c r="D53" s="10">
         <v>96</v>
       </c>
-      <c r="D53" s="11">
+      <c r="E53" s="11">
         <v>1.0405092592592593E-2</v>
       </c>
-      <c r="E53" s="10">
+      <c r="F53" s="10">
         <v>63</v>
       </c>
-      <c r="F53" s="10" t="s">
+      <c r="G53" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="G53" s="10">
+      <c r="H53" s="10">
         <v>43</v>
       </c>
-      <c r="H53" s="10">
+      <c r="I53" s="10">
         <v>79.489999999999995</v>
       </c>
-      <c r="I53" s="10" t="s">
+      <c r="J53" s="10" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="54" spans="1:9">
-      <c r="A54" s="12" t="s">
+    <row r="54" spans="1:10">
+      <c r="A54" s="10">
+        <v>51</v>
+      </c>
+      <c r="B54" s="12" t="s">
         <v>175</v>
       </c>
-      <c r="B54" s="12" t="s">
+      <c r="C54" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C54" s="12">
+      <c r="D54" s="12">
         <v>191</v>
       </c>
-      <c r="D54" s="13">
+      <c r="E54" s="13">
         <v>1.3680555555555555E-2</v>
       </c>
-      <c r="E54" s="12">
+      <c r="F54" s="12">
         <v>63</v>
       </c>
-      <c r="F54" s="12" t="s">
+      <c r="G54" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="G54" s="12">
+      <c r="H54" s="12">
         <v>40</v>
       </c>
-      <c r="H54" s="12">
+      <c r="I54" s="12">
         <v>60.1</v>
       </c>
-      <c r="I54" s="12" t="s">
+      <c r="J54" s="12" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="55" spans="1:9">
-      <c r="A55" s="10" t="s">
+    <row r="55" spans="1:10">
+      <c r="A55" s="12">
+        <v>52</v>
+      </c>
+      <c r="B55" s="10" t="s">
         <v>177</v>
       </c>
-      <c r="B55" s="10" t="s">
+      <c r="C55" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="C55" s="10">
+      <c r="D55" s="10">
         <v>131</v>
       </c>
-      <c r="D55" s="11">
+      <c r="E55" s="11">
         <v>1.3541666666666667E-2</v>
       </c>
-      <c r="E55" s="10">
+      <c r="F55" s="10">
         <v>63</v>
       </c>
-      <c r="F55" s="10" t="s">
+      <c r="G55" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="G55" s="10">
+      <c r="H55" s="10">
         <v>42</v>
       </c>
-      <c r="H55" s="10">
+      <c r="I55" s="10">
         <v>53.08</v>
       </c>
-      <c r="I55" s="10" t="s">
+      <c r="J55" s="10" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="56" spans="1:9">
-      <c r="A56" s="10" t="s">
+    <row r="56" spans="1:10">
+      <c r="A56" s="10">
+        <v>53</v>
+      </c>
+      <c r="B56" s="10" t="s">
         <v>179</v>
       </c>
-      <c r="B56" s="10" t="s">
+      <c r="C56" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="C56" s="10">
+      <c r="D56" s="10">
         <v>153</v>
       </c>
-      <c r="D56" s="11">
+      <c r="E56" s="11">
         <v>1.2650462962962962E-2</v>
       </c>
-      <c r="E56" s="10">
+      <c r="F56" s="10">
         <v>63</v>
       </c>
-      <c r="F56" s="10" t="s">
+      <c r="G56" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="G56" s="10">
+      <c r="H56" s="10">
         <v>43</v>
       </c>
-      <c r="H56" s="10">
+      <c r="I56" s="10">
         <v>59.84</v>
       </c>
-      <c r="I56" s="10" t="s">
+      <c r="J56" s="10" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="57" spans="1:9">
-      <c r="A57" s="12" t="s">
+    <row r="57" spans="1:10">
+      <c r="A57" s="12">
+        <v>54</v>
+      </c>
+      <c r="B57" s="12" t="s">
         <v>181</v>
       </c>
-      <c r="B57" s="12" t="s">
+      <c r="C57" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C57" s="12">
+      <c r="D57" s="12">
         <v>165</v>
       </c>
-      <c r="D57" s="13">
+      <c r="E57" s="13">
         <v>1.3460648148148149E-2</v>
       </c>
-      <c r="E57" s="12">
+      <c r="F57" s="12">
         <v>63</v>
       </c>
-      <c r="F57" s="12" t="s">
+      <c r="G57" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="G57" s="12">
+      <c r="H57" s="12">
         <v>42</v>
       </c>
-      <c r="H57" s="12">
+      <c r="I57" s="12">
         <v>61.91</v>
       </c>
-      <c r="I57" s="12" t="s">
+      <c r="J57" s="12" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="58" spans="1:9">
-      <c r="A58" s="12" t="s">
+    <row r="58" spans="1:10">
+      <c r="A58" s="10">
+        <v>55</v>
+      </c>
+      <c r="B58" s="12" t="s">
         <v>183</v>
       </c>
-      <c r="B58" s="12" t="s">
+      <c r="C58" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C58" s="12">
+      <c r="D58" s="12">
         <v>123</v>
       </c>
-      <c r="D58" s="13">
+      <c r="E58" s="13">
         <v>1.1400462962962963E-2</v>
       </c>
-      <c r="E58" s="12">
+      <c r="F58" s="12">
         <v>63</v>
       </c>
-      <c r="F58" s="12" t="s">
+      <c r="G58" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="G58" s="12">
+      <c r="H58" s="12">
         <v>33</v>
       </c>
-      <c r="H58" s="12">
+      <c r="I58" s="12">
         <v>66.7</v>
       </c>
-      <c r="I58" s="12" t="s">
+      <c r="J58" s="12" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="59" spans="1:9">
-      <c r="A59" s="12" t="s">
+    <row r="59" spans="1:10">
+      <c r="A59" s="12">
+        <v>56</v>
+      </c>
+      <c r="B59" s="12" t="s">
         <v>185</v>
       </c>
-      <c r="B59" s="12" t="s">
+      <c r="C59" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C59" s="12">
+      <c r="D59" s="12">
         <v>343</v>
       </c>
-      <c r="D59" s="13">
+      <c r="E59" s="13">
         <v>3.1851851851851853E-2</v>
       </c>
-      <c r="E59" s="12">
+      <c r="F59" s="12">
         <v>63</v>
       </c>
-      <c r="F59" s="12" t="s">
+      <c r="G59" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="G59" s="12">
+      <c r="H59" s="12">
         <v>41</v>
       </c>
-      <c r="H59" s="12">
+      <c r="I59" s="12">
         <v>46.85</v>
       </c>
-      <c r="I59" s="12" t="s">
+      <c r="J59" s="12" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="60" spans="1:9">
-      <c r="A60" s="10" t="s">
+    <row r="60" spans="1:10">
+      <c r="A60" s="10">
+        <v>57</v>
+      </c>
+      <c r="B60" s="10" t="s">
         <v>187</v>
       </c>
-      <c r="B60" s="10" t="s">
+      <c r="C60" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="C60" s="10">
+      <c r="D60" s="10">
         <v>135</v>
       </c>
-      <c r="D60" s="11">
+      <c r="E60" s="11">
         <v>1.1342592592592593E-2</v>
       </c>
-      <c r="E60" s="10">
+      <c r="F60" s="10">
         <v>63</v>
       </c>
-      <c r="F60" s="10" t="s">
+      <c r="G60" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="G60" s="10">
+      <c r="H60" s="10">
         <v>43</v>
       </c>
-      <c r="H60" s="10">
+      <c r="I60" s="10">
         <v>56.33</v>
       </c>
-      <c r="I60" s="10" t="s">
+      <c r="J60" s="10" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="61" spans="1:9">
-      <c r="A61" s="10" t="s">
+    <row r="61" spans="1:10">
+      <c r="A61" s="12">
+        <v>58</v>
+      </c>
+      <c r="B61" s="10" t="s">
         <v>189</v>
       </c>
-      <c r="B61" s="10" t="s">
+      <c r="C61" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="C61" s="10">
+      <c r="D61" s="10">
         <v>78</v>
       </c>
-      <c r="D61" s="11">
+      <c r="E61" s="11">
         <v>7.5810185185185182E-3</v>
       </c>
-      <c r="E61" s="10">
+      <c r="F61" s="10">
         <v>63</v>
       </c>
-      <c r="F61" s="10" t="s">
+      <c r="G61" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="G61" s="10">
+      <c r="H61" s="10">
         <v>43</v>
       </c>
-      <c r="H61" s="10">
+      <c r="I61" s="10">
         <v>68.7</v>
       </c>
-      <c r="I61" s="10" t="s">
+      <c r="J61" s="10" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="62" spans="1:9">
-      <c r="A62" s="10" t="s">
+    <row r="62" spans="1:10">
+      <c r="A62" s="10">
+        <v>59</v>
+      </c>
+      <c r="B62" s="10" t="s">
         <v>191</v>
       </c>
-      <c r="B62" s="10" t="s">
+      <c r="C62" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="C62" s="10">
+      <c r="D62" s="10">
         <v>58</v>
       </c>
-      <c r="D62" s="11">
+      <c r="E62" s="11">
         <v>8.0439814814814818E-3</v>
       </c>
-      <c r="E62" s="10">
+      <c r="F62" s="10">
         <v>63</v>
       </c>
-      <c r="F62" s="10" t="s">
+      <c r="G62" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="G62" s="10">
+      <c r="H62" s="10">
         <v>42</v>
       </c>
-      <c r="H62" s="10">
+      <c r="I62" s="10">
         <v>56.03</v>
       </c>
-      <c r="I62" s="10" t="s">
+      <c r="J62" s="10" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="63" spans="1:9">
-      <c r="A63" s="12" t="s">
+    <row r="63" spans="1:10">
+      <c r="A63" s="12">
+        <v>60</v>
+      </c>
+      <c r="B63" s="12" t="s">
         <v>193</v>
       </c>
-      <c r="B63" s="12" t="s">
+      <c r="C63" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C63" s="12">
+      <c r="D63" s="12">
         <v>118</v>
       </c>
-      <c r="D63" s="13">
+      <c r="E63" s="13">
         <v>1.0868055555555556E-2</v>
       </c>
-      <c r="E63" s="12">
+      <c r="F63" s="12">
         <v>40</v>
       </c>
-      <c r="F63" s="12" t="s">
+      <c r="G63" s="12" t="s">
         <v>194</v>
       </c>
-      <c r="G63" s="12">
+      <c r="H63" s="12">
         <v>31</v>
       </c>
-      <c r="H63" s="12">
+      <c r="I63" s="12">
         <v>70.930000000000007</v>
       </c>
-      <c r="I63" s="12" t="s">
+      <c r="J63" s="12" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="64" spans="1:9">
-      <c r="A64" s="12" t="s">
+    <row r="64" spans="1:10">
+      <c r="A64" s="10">
+        <v>61</v>
+      </c>
+      <c r="B64" s="12" t="s">
         <v>196</v>
       </c>
-      <c r="B64" s="12" t="s">
+      <c r="C64" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C64" s="12">
+      <c r="D64" s="12">
         <v>63</v>
       </c>
-      <c r="D64" s="13">
+      <c r="E64" s="13">
         <v>1.0555555555555556E-2</v>
       </c>
-      <c r="E64" s="12">
+      <c r="F64" s="12">
         <v>63</v>
       </c>
-      <c r="F64" s="12" t="s">
+      <c r="G64" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="G64" s="12">
+      <c r="H64" s="12">
         <v>31</v>
       </c>
-      <c r="H64" s="12">
+      <c r="I64" s="12">
         <v>57.83</v>
       </c>
-      <c r="I64" s="12" t="s">
+      <c r="J64" s="12" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="65" spans="4:4">
-      <c r="D65" s="16"/>
-    </row>
-    <row r="66" spans="4:4">
-      <c r="D66" s="16"/>
-    </row>
-    <row r="67" spans="4:4">
-      <c r="D67" s="16"/>
-    </row>
-    <row r="68" spans="4:4">
-      <c r="D68" s="16"/>
-    </row>
-    <row r="69" spans="4:4">
-      <c r="D69" s="16"/>
-    </row>
-    <row r="70" spans="4:4">
-      <c r="D70" s="16"/>
-    </row>
-    <row r="71" spans="4:4">
-      <c r="D71" s="16"/>
+    <row r="65" spans="5:5">
+      <c r="E65" s="16"/>
+    </row>
+    <row r="66" spans="5:5">
+      <c r="E66" s="16"/>
+    </row>
+    <row r="67" spans="5:5">
+      <c r="E67" s="16"/>
+    </row>
+    <row r="68" spans="5:5">
+      <c r="E68" s="16"/>
+    </row>
+    <row r="69" spans="5:5">
+      <c r="E69" s="16"/>
+    </row>
+    <row r="70" spans="5:5">
+      <c r="E70" s="16"/>
+    </row>
+    <row r="71" spans="5:5">
+      <c r="E71" s="16"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -32552,15 +32743,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100309D7ACAE19AEA4188E74FC911064806" ma:contentTypeVersion="13" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="ae129f4de42350f471a77453777943df">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6656c2dc-2965-4315-a8fd-a4d95559af9c" xmlns:ns3="771465c8-566f-4c1b-b214-95c896f401f4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="49ad4b641c41180eb1c519bf4e5a8e65" ns2:_="" ns3:_="">
     <xsd:import namespace="6656c2dc-2965-4315-a8fd-a4d95559af9c"/>
@@ -32761,6 +32943,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{203948C1-2CCB-4F17-8271-4735FF7E256D}">
   <ds:schemaRefs>
@@ -32773,14 +32964,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1CD06BC1-8140-4AD3-BDED-91AD01E5356E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67F3D48C-D3CB-49AA-A8AD-4A78A78029A1}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -32797,4 +32980,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1CD06BC1-8140-4AD3-BDED-91AD01E5356E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>